<commit_message>
Record UI login-blocked on 9481-9499 pending prototype GUI secrets
Select Receipts was not attempted. KIMCO_PROTOTYPE_USERNAME and
KIMCO_PROTOTYPE_PASSWORD are absent. Headers were left unchanged.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -579,7 +579,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -637,7 +637,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -695,7 +695,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -753,7 +753,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -811,7 +811,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -869,7 +869,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -927,7 +927,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -985,7 +985,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Header created. Lines blocked/405: API cannot Select Receipts until Editable is on; do not type Add Item. Fees recorded in Fees and surcharges (not PPV). Attach status=no-pdf-on-vm.</t>
+          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Note UI secrets still invisible on this run; relaunch required
9481-9499 remain login-blocked. Select Receipts was not attempted.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -614,7 +614,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -672,7 +672,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -730,7 +730,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -788,7 +788,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -904,7 +904,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -962,7 +962,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD absent. Select Receipts not attempted. Header left as created. No void/delete.</t>
+          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">

</xml_diff>

<commit_message>
Record prototype GUI Select Receipts for 9484-9486
9484 Purvis: selected PO58556 receipt qty 10 and posted F-Fees & Surcharges 27.12.
9485-9486 Capital PO 58634: HOLD-no-receipts. No lines invented.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -730,7 +730,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Receipt selected from PO58556-01 qty 10, fee 27.12 posted. Receipts: PO58556-01 slip 23016800 qty 10 part TBL00005. Fees posted: F-Fees &amp; Surcharges 27.12 Total Freight In. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -781,14 +781,14 @@
       <c r="E6" s="2" t="n">
         <v>403</v>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>HOLD-no-receipts. Receipts: none - PO 58634 has no receipts in prototype. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -839,14 +839,14 @@
       <c r="E7" s="2" t="n">
         <v>940</v>
       </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>HOLD-no-receipts. Receipts: none - PO 58634 has no receipts in prototype. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">

</xml_diff>

<commit_message>
Record GUI results for 9488, 9490, 9494-9496, 9498
O'Neal 9490 and EMJ 9498 Select Receipts succeeded.
Legacy 9494-9496 and Willbanks 9488 are HOLD-no-receipts.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -730,7 +730,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Receipt selected from PO58556-01 qty 10, fee 27.12 posted. Receipts: PO58556-01 slip 23016800 qty 10 part TBL00005. Fees posted: F-Fees &amp; Surcharges 27.12 Total Freight In. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Receipt selected from PO58556-01 qty 10, fee 27.12 posted Receipts: PO58556-01 slip 23016800 qty 10 part TBL00005. Fees posted: F-Fees &amp; Surcharges 27.12 Total Freight In. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -788,7 +788,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Receipts: none - PO 58634 has no receipts in prototype. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>HOLD-no-receipts Receipts: none - PO 58634 has no receipts in prototype. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Receipts: none - PO 58634 has no receipts in prototype. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>HOLD-no-receipts Receipts: none - PO 58634 has no receipts in prototype. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -955,14 +955,14 @@
       <c r="E9" s="2" t="n">
         <v>3347.97</v>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>HOLD-no-receipts. Select Receipts showed no matching uninvoiced receipts. Did not invent lines. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: PO58799 PL-0.25 X 60 X 120-A572 qty 5 slip 84615375. No $0 freight charge. Invoice amount 2278.11 matches. Receipts: PO58799-01 qty 5. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -1303,14 +1303,14 @@
       <c r="E15" s="2" t="n">
         <v>2545</v>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>HOLD-no-receipts. Select Receipts showed no matching uninvoiced receipts. Did not invent lines. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1361,14 +1361,14 @@
       <c r="E16" s="2" t="n">
         <v>2140</v>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>HOLD-no-receipts. Select Receipts showed no matching uninvoiced receipts. Did not invent lines. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1419,14 +1419,14 @@
       <c r="E17" s="2" t="n">
         <v>856</v>
       </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>HOLD-no-receipts. Select Receipts showed no matching uninvoiced receipts. Did not invent lines. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: both PO58810 RB-4.00-6061 receipts 13ea + 35ea slip S812773. Amount 393.60 vs verification 393.62 (2-cent rounding). No fees. Receipts: PO58810-01 qty 13; PO58810-02 qty 35. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">

</xml_diff>

<commit_message>
Record GUI Select Receipts for 9491, 9493, 9497, 9499
O'Neal 9491 selected only the 8/3 tread-plate receipt.
Fastenal 9493 and Eastern Metal 9497 posted shipping as F-Fees & Surcharges.
Crosslink 9499 packaging 12.40 is Fees, not PPV; no invented unreceived line.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -730,7 +730,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Receipt selected from PO58556-01 qty 10, fee 27.12 posted Receipts: PO58556-01 slip 23016800 qty 10 part TBL00005. Fees posted: F-Fees &amp; Surcharges 27.12 Total Freight In. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Receipt selected from PO58556-01 qty 10, fee 27.12 posted Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -788,7 +788,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts Receipts: none - PO 58634 has no receipts in prototype. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>HOLD-no-receipts Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts Receipts: none - PO 58634 has no receipts in prototype. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>HOLD-no-receipts Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -962,7 +962,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts showed no matching uninvoiced receipts. Did not invent lines. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Select Receipts showed no items for PO 58383 (MARMON-KEYSTONE in prototype) Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58799 PL-0.25 X 60 X 120-A572 qty 5 slip 84615375. No $0 freight charge. Invoice amount 2278.11 matches. Receipts: PO58799-01 qty 5. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Receipt added for part PL-0.25 X 60 X 120-A572, qty 5, slip 84615375 Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: only 8/3 slip 84623830 TP-0.125 x 60 x 120-A36 qty 20. Did not select 8/5 PL-0.375. Amount 5580.96 matches. No $0 freight. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: all 3 PO58764 receipts (TXFT499769). Posted F-Fees &amp; Surcharges 122.69 Shipping &amp; Handling (not PPV). Amount 424.89 vs verification 424.88. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts showed no matching uninvoiced receipts. Did not invent lines. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Select Receipts showed no items for PO 58821 Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts showed no matching uninvoiced receipts. Did not invent lines. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Select Receipts showed no items for PO 58717 Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts showed no matching uninvoiced receipts. Did not invent lines. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Select Receipts showed no items for PO 58742 Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: both PO58814 receipts slip G62282. Posted F-Fees &amp; Surcharges 60.00 SHIPPING &amp; HANDLING SURCHARGE (not PPV). Amount 1681.19 vs verification 1681.31 (PO price rounding). Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both PO58810 RB-4.00-6061 receipts 13ea + 35ea slip S812773. Amount 393.60 vs verification 393.62 (2-cent rounding). No fees. Receipts: PO58810-01 qty 13; PO58810-02 qty 35. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Both receipts added: 13ea and 35ea RB-4.00-6061, slip S812773, total qty 48 Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: PO58723-02 qty 1 and PO58723-03 qty 2. Did not Add Item for unreceived line 01. Posted F-Fees &amp; Surcharges 12.40 Packaging/Shop Supplies Recovery (NOT PPV). Amount 670.36 vs verification 1252.18 because line 01 has no receipt. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">

</xml_diff>

<commit_message>
Record prototype GUI outcomes for AP invoices 9481-9499
Select Receipts completed on all 19 batch-671 headers. HOLD-no-receipts
where the prototype had no matching receipts. Fees posted as F-Fees &
Surcharges only (9486/9499 shop supplies and packaging are not PPV).

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: slip 106081 qty 38+58=96 of A-04421-000 @ 108.66. Invoice amount 10431.36 matches. No fees. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -614,7 +614,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: 5913K74 qty 10 and 91263A232 qty 5. Did not Add Item for unreceived 8701K65. Posted F-Fees &amp; Surcharges 42.17 Shipping (not PPV). Amount 205.52 vs verification 489.14 because line 01 has no receipt. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -672,7 +672,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: all 8 PO58826 receipts slip 3262728-02. Posted F-Fees &amp; Surcharges 38.83 Shipping (not PPV). Amount 467.22 matches. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -730,7 +730,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Receipt selected from PO58556-01 qty 10, fee 27.12 posted Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Select Receipts: PO58556-01 qty 10 slip 23016800. Posted F-Fees &amp; Surcharges 27.12 Total Freight In (not PPV). Amount 480.05 matches. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -788,7 +788,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Did not invent lines or freight. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Shop supplies 25.00 would be F-Fees &amp; Surcharges never PPV, but no receipts so no invented lines/charges. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -904,7 +904,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: both 7/30 slip 186040-3 (S0264-1 qty 12, S0264-4 qty 24). No PPV added (1906.68 vs invoice 1828.08). Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -962,7 +962,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts showed no items for PO 58383 (MARMON-KEYSTONE in prototype) Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58383 (prototype vendor Marmon-Keystone; only historical receipt already invoiced). Did not invent lines. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: slip 331201 two A-02393-000 qty 42+42 plus A-09128-000* lid qty 30. Skipped 8/4 and negative qty. Amount 13404.84 matches. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Receipt added for part PL-0.25 X 60 X 120-A572, qty 5, slip 84615375 Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Select Receipts: PO58799 PL-0.25 X 60 X 120-A572 qty 5 slip 84615375. No $0 freight charge. Amount 2278.11 matches. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: only 8/3 slip 84623830 TP-0.125 x 60 x 120-A36 qty 20. Did not select 8/5 PL-0.375. Amount 5580.96 matches. No $0 freight. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Select Receipts: only 8/3 slip 84623830 TP-0.125 x 60 x 120-A36 qty 20. Did not select 8/5 PL-0.375. Amount 5580.96 matches. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>UI login-blocked: this run still cannot see KIMCO_PROTOTYPE_USERNAME / KIMCO_PROTOTYPE_PASSWORD (also checked KIMCO_USERNAME / KIMCO_PASSWORD). Relaunch on the beave89atm/ap-clerk environment so the new secrets inject. Select Receipts not attempted. Did not invent credentials or use the API key as a GUI password.</t>
+          <t>Select Receipts: all 15 PO58749 receipts. Posted F-Fees &amp; Surcharges 124.83 Shipping &amp; Handling (not PPV). Amount 2620.08 matches. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 3 PO58764 receipts (TXFT499769). Posted F-Fees &amp; Surcharges 122.69 Shipping &amp; Handling (not PPV). Amount 424.89 vs verification 424.88. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Select Receipts: all 3 PO58764 receipts slips TXFT499769. Posted F-Fees &amp; Surcharges 122.69 Shipping &amp; Handling (not PPV). Amount 424.89 vs verification 424.88. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts showed no items for PO 58821 Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58821. Did not invent freight 700. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts showed no items for PO 58717 Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58717. Did not invent freight 500. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts showed no items for PO 58742 Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58742. Did not invent freight 200. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both PO58814 receipts slip G62282. Posted F-Fees &amp; Surcharges 60.00 SHIPPING &amp; HANDLING SURCHARGE (not PPV). Amount 1681.19 vs verification 1681.31 (PO price rounding). Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Select Receipts: both PO58814 receipts slip G62282. Posted F-Fees &amp; Surcharges 60.00 SHIPPING &amp; HANDLING SURCHARGE (not PPV). Amount 1681.19 vs verification 1681.31. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Both receipts added: 13ea and 35ea RB-4.00-6061, slip S812773, total qty 48 Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Select Receipts: both PO58810 RB-4.00-6061 receipts 13+35 slip S812773. Amount 393.60 vs verification 393.62. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58723-02 qty 1 and PO58723-03 qty 2. Did not Add Item for unreceived line 01. Posted F-Fees &amp; Surcharges 12.40 Packaging/Shop Supplies Recovery (NOT PPV). Amount 670.36 vs verification 1252.18 because line 01 has no receipt. Attach=no-pdf. GUI Select Receipts on prototype only; did not void/recreate.</t>
+          <t>Select Receipts: PO58723-02 qty 1 and PO58723-03 qty 2. Did not Add Item for unreceived line 01. Posted F-Fees &amp; Surcharges 12.40 Packaging/Shop Supplies Recovery (NOT PPV). Amount 670.36 vs verification 1252.18. Attach=no-pdf.</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">

</xml_diff>

<commit_message>
Record Outlook mailbox login-blocked for AP attach 9481-9499
accountspayable@kannonmfg.com is recognized in Outlook on the web, but this environment has no mailbox password or Graph secrets. No vendor PDFs were downloaded or committed.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: slip 106081 qty 38+58=96 of A-04421-000 @ 108.66. Invoice amount 10431.36 matches. No fees. Attach=no-pdf.</t>
+          <t>Select Receipts: slip 106081 qty 38+58=96 of A-04421-000 @ 108.66. Invoice amount 10431.36 matches. No fees. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -579,7 +579,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: 5913K74 qty 10 and 91263A232 qty 5. Did not Add Item for unreceived 8701K65. Posted F-Fees &amp; Surcharges 42.17 Shipping (not PPV). Amount 205.52 vs verification 489.14 because line 01 has no receipt. Attach=no-pdf.</t>
+          <t>Select Receipts: 5913K74 qty 10 and 91263A232 qty 5. Did not Add Item for unreceived 8701K65. Posted F-Fees &amp; Surcharges 42.17 Shipping (not PPV). Amount 205.52 vs verification 489.14 because line 01 has no receipt. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -637,7 +637,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 8 PO58826 receipts slip 3262728-02. Posted F-Fees &amp; Surcharges 38.83 Shipping (not PPV). Amount 467.22 matches. Attach=no-pdf.</t>
+          <t>Select Receipts: all 8 PO58826 receipts slip 3262728-02. Posted F-Fees &amp; Surcharges 38.83 Shipping (not PPV). Amount 467.22 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -695,7 +695,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58556-01 qty 10 slip 23016800. Posted F-Fees &amp; Surcharges 27.12 Total Freight In (not PPV). Amount 480.05 matches. Attach=no-pdf.</t>
+          <t>Select Receipts: PO58556-01 qty 10 slip 23016800. Posted F-Fees &amp; Surcharges 27.12 Total Freight In (not PPV). Amount 480.05 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -753,7 +753,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Did not invent lines or freight. Attach=no-pdf.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Did not invent lines or freight. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -811,7 +811,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Shop supplies 25.00 would be F-Fees &amp; Surcharges never PPV, but no receipts so no invented lines/charges. Attach=no-pdf.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Shop supplies 25.00 would be F-Fees &amp; Surcharges never PPV, but no receipts so no invented lines/charges. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -869,7 +869,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both 7/30 slip 186040-3 (S0264-1 qty 12, S0264-4 qty 24). No PPV added (1906.68 vs invoice 1828.08). Attach=no-pdf.</t>
+          <t>Select Receipts: both 7/30 slip 186040-3 (S0264-1 qty 12, S0264-4 qty 24). No PPV added (1906.68 vs invoice 1828.08). Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -927,7 +927,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58383 (prototype vendor Marmon-Keystone; only historical receipt already invoiced). Did not invent lines. Attach=no-pdf.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58383 (prototype vendor Marmon-Keystone; only historical receipt already invoiced). Did not invent lines. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -985,7 +985,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: slip 331201 two A-02393-000 qty 42+42 plus A-09128-000* lid qty 30. Skipped 8/4 and negative qty. Amount 13404.84 matches. Attach=no-pdf.</t>
+          <t>Select Receipts: slip 331201 two A-02393-000 qty 42+42 plus A-09128-000* lid qty 30. Skipped 8/4 and negative qty. Amount 13404.84 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58799 PL-0.25 X 60 X 120-A572 qty 5 slip 84615375. No $0 freight charge. Amount 2278.11 matches. Attach=no-pdf.</t>
+          <t>Select Receipts: PO58799 PL-0.25 X 60 X 120-A572 qty 5 slip 84615375. No $0 freight charge. Amount 2278.11 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: only 8/3 slip 84623830 TP-0.125 x 60 x 120-A36 qty 20. Did not select 8/5 PL-0.375. Amount 5580.96 matches. Attach=no-pdf.</t>
+          <t>Select Receipts: only 8/3 slip 84623830 TP-0.125 x 60 x 120-A36 qty 20. Did not select 8/5 PL-0.375. Amount 5580.96 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 15 PO58749 receipts. Posted F-Fees &amp; Surcharges 124.83 Shipping &amp; Handling (not PPV). Amount 2620.08 matches. Attach=no-pdf.</t>
+          <t>Select Receipts: all 15 PO58749 receipts. Posted F-Fees &amp; Surcharges 124.83 Shipping &amp; Handling (not PPV). Amount 2620.08 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 3 PO58764 receipts slips TXFT499769. Posted F-Fees &amp; Surcharges 122.69 Shipping &amp; Handling (not PPV). Amount 424.89 vs verification 424.88. Attach=no-pdf.</t>
+          <t>Select Receipts: all 3 PO58764 receipts slips TXFT499769. Posted F-Fees &amp; Surcharges 122.69 Shipping &amp; Handling (not PPV). Amount 424.89 vs verification 424.88. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58821. Did not invent freight 700. Attach=no-pdf.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58821. Did not invent freight 700. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58717. Did not invent freight 500. Attach=no-pdf.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58717. Did not invent freight 500. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58742. Did not invent freight 200. Attach=no-pdf.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58742. Did not invent freight 200. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both PO58814 receipts slip G62282. Posted F-Fees &amp; Surcharges 60.00 SHIPPING &amp; HANDLING SURCHARGE (not PPV). Amount 1681.19 vs verification 1681.31. Attach=no-pdf.</t>
+          <t>Select Receipts: both PO58814 receipts slip G62282. Posted F-Fees &amp; Surcharges 60.00 SHIPPING &amp; HANDLING SURCHARGE (not PPV). Amount 1681.19 vs verification 1681.31. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both PO58810 RB-4.00-6061 receipts 13+35 slip S812773. Amount 393.60 vs verification 393.62. Attach=no-pdf.</t>
+          <t>Select Receipts: both PO58810 RB-4.00-6061 receipts 13+35 slip S812773. Amount 393.60 vs verification 393.62. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58723-02 qty 1 and PO58723-03 qty 2. Did not Add Item for unreceived line 01. Posted F-Fees &amp; Surcharges 12.40 Packaging/Shop Supplies Recovery (NOT PPV). Amount 670.36 vs verification 1252.18. Attach=no-pdf.</t>
+          <t>Select Receipts: PO58723-02 qty 1 and PO58723-03 qty 2. Did not Add Item for unreceived line 01. Posted F-Fees &amp; Surcharges 12.40 Packaging/Shop Supplies Recovery (NOT PPV). Amount 670.36 vs verification 1252.18. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>no-pdf</t>
+          <t>login-blocked</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record Outlook password rejection for AP attach 9481-9499
OUTLOOK_AP_PASSWORD is present but Microsoft rejected it for
accountspayable@kannonmfg.com. No other mailbox was opened.
No vendor PDFs were downloaded or committed.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: slip 106081 qty 38+58=96 of A-04421-000 @ 108.66. Invoice amount 10431.36 matches. No fees. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: slip 106081 qty 38+58=96 of A-04421-000 @ 108.66. Invoice amount 10431.36 matches. No fees. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -614,7 +614,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: 5913K74 qty 10 and 91263A232 qty 5. Did not Add Item for unreceived 8701K65. Posted F-Fees &amp; Surcharges 42.17 Shipping (not PPV). Amount 205.52 vs verification 489.14 because line 01 has no receipt. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: 5913K74 qty 10 and 91263A232 qty 5. Did not Add Item for unreceived 8701K65. Posted F-Fees &amp; Surcharges 42.17 Shipping (not PPV). Amount 205.52 vs verification 489.14 because line 01 has no receipt. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -672,7 +672,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 8 PO58826 receipts slip 3262728-02. Posted F-Fees &amp; Surcharges 38.83 Shipping (not PPV). Amount 467.22 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: all 8 PO58826 receipts slip 3262728-02. Posted F-Fees &amp; Surcharges 38.83 Shipping (not PPV). Amount 467.22 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -730,7 +730,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58556-01 qty 10 slip 23016800. Posted F-Fees &amp; Surcharges 27.12 Total Freight In (not PPV). Amount 480.05 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: PO58556-01 qty 10 slip 23016800. Posted F-Fees &amp; Surcharges 27.12 Total Freight In (not PPV). Amount 480.05 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -788,7 +788,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Did not invent lines or freight. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Did not invent lines or freight. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Shop supplies 25.00 would be F-Fees &amp; Surcharges never PPV, but no receipts so no invented lines/charges. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Shop supplies 25.00 would be F-Fees &amp; Surcharges never PPV, but no receipts so no invented lines/charges. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -904,7 +904,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both 7/30 slip 186040-3 (S0264-1 qty 12, S0264-4 qty 24). No PPV added (1906.68 vs invoice 1828.08). Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: both 7/30 slip 186040-3 (S0264-1 qty 12, S0264-4 qty 24). No PPV added (1906.68 vs invoice 1828.08). Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -962,7 +962,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58383 (prototype vendor Marmon-Keystone; only historical receipt already invoiced). Did not invent lines. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58383 (prototype vendor Marmon-Keystone; only historical receipt already invoiced). Did not invent lines. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: slip 331201 two A-02393-000 qty 42+42 plus A-09128-000* lid qty 30. Skipped 8/4 and negative qty. Amount 13404.84 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: slip 331201 two A-02393-000 qty 42+42 plus A-09128-000* lid qty 30. Skipped 8/4 and negative qty. Amount 13404.84 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58799 PL-0.25 X 60 X 120-A572 qty 5 slip 84615375. No $0 freight charge. Amount 2278.11 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: PO58799 PL-0.25 X 60 X 120-A572 qty 5 slip 84615375. No $0 freight charge. Amount 2278.11 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: only 8/3 slip 84623830 TP-0.125 x 60 x 120-A36 qty 20. Did not select 8/5 PL-0.375. Amount 5580.96 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: only 8/3 slip 84623830 TP-0.125 x 60 x 120-A36 qty 20. Did not select 8/5 PL-0.375. Amount 5580.96 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 15 PO58749 receipts. Posted F-Fees &amp; Surcharges 124.83 Shipping &amp; Handling (not PPV). Amount 2620.08 matches. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: all 15 PO58749 receipts. Posted F-Fees &amp; Surcharges 124.83 Shipping &amp; Handling (not PPV). Amount 2620.08 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 3 PO58764 receipts slips TXFT499769. Posted F-Fees &amp; Surcharges 122.69 Shipping &amp; Handling (not PPV). Amount 424.89 vs verification 424.88. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: all 3 PO58764 receipts slips TXFT499769. Posted F-Fees &amp; Surcharges 122.69 Shipping &amp; Handling (not PPV). Amount 424.89 vs verification 424.88. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58821. Did not invent freight 700. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58821. Did not invent freight 700. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58717. Did not invent freight 500. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58717. Did not invent freight 500. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58742. Did not invent freight 200. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58742. Did not invent freight 200. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both PO58814 receipts slip G62282. Posted F-Fees &amp; Surcharges 60.00 SHIPPING &amp; HANDLING SURCHARGE (not PPV). Amount 1681.19 vs verification 1681.31. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: both PO58814 receipts slip G62282. Posted F-Fees &amp; Surcharges 60.00 SHIPPING &amp; HANDLING SURCHARGE (not PPV). Amount 1681.19 vs verification 1681.31. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both PO58810 RB-4.00-6061 receipts 13+35 slip S812773. Amount 393.60 vs verification 393.62. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: both PO58810 RB-4.00-6061 receipts 13+35 slip S812773. Amount 393.60 vs verification 393.62. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58723-02 qty 1 and PO58723-03 qty 2. Did not Add Item for unreceived line 01. Posted F-Fees &amp; Surcharges 12.40 Packaging/Shop Supplies Recovery (NOT PPV). Amount 670.36 vs verification 1252.18. Attach=login-blocked: Outlook recognized accountspayable@kannonmfg.com but OUTLOOK_AP_PASSWORD is absent; no PDF downloaded.</t>
+          <t>Select Receipts: PO58723-02 qty 1 and PO58723-03 qty 2. Did not Add Item for unreceived line 01. Posted F-Fees &amp; Surcharges 12.40 Packaging/Shop Supplies Recovery (NOT PPV). Amount 670.36 vs verification 1252.18. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">

</xml_diff>

<commit_message>
Record Graph header attach for AP invoices 9481-9499
Vendor PDFs were pulled from accountspayable@kannonmfg.com via Microsoft Graph and uploaded on the existing prototype invoice headers. No PDFs or secrets are committed.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: slip 106081 qty 38+58=96 of A-04421-000 @ 108.66. Invoice amount 10431.36 matches. No fees. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: slip 106081 qty 38+58=96 of A-04421-000 @ 108.66. Invoice amount 10431.36 matches. No fees. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -579,7 +579,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: 5913K74 qty 10 and 91263A232 qty 5. Did not Add Item for unreceived 8701K65. Posted F-Fees &amp; Surcharges 42.17 Shipping (not PPV). Amount 205.52 vs verification 489.14 because line 01 has no receipt. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: 5913K74 qty 10 and 91263A232 qty 5. Did not Add Item for unreceived 8701K65. Posted F-Fees &amp; Surcharges 42.17 Shipping (not PPV). Amount 205.52 vs verification 489.14 because line 01 has no receipt. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -637,7 +637,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 8 PO58826 receipts slip 3262728-02. Posted F-Fees &amp; Surcharges 38.83 Shipping (not PPV). Amount 467.22 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: all 8 PO58826 receipts slip 3262728-02. Posted F-Fees &amp; Surcharges 38.83 Shipping (not PPV). Amount 467.22 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -695,7 +695,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58556-01 qty 10 slip 23016800. Posted F-Fees &amp; Surcharges 27.12 Total Freight In (not PPV). Amount 480.05 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: PO58556-01 qty 10 slip 23016800. Posted F-Fees &amp; Surcharges 27.12 Total Freight In (not PPV). Amount 480.05 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -753,7 +753,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Did not invent lines or freight. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Did not invent lines or freight. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -811,7 +811,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Shop supplies 25.00 would be F-Fees &amp; Surcharges never PPV, but no receipts so no invented lines/charges. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Shop supplies 25.00 would be F-Fees &amp; Surcharges never PPV, but no receipts so no invented lines/charges. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -869,7 +869,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both 7/30 slip 186040-3 (S0264-1 qty 12, S0264-4 qty 24). No PPV added (1906.68 vs invoice 1828.08). Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: both 7/30 slip 186040-3 (S0264-1 qty 12, S0264-4 qty 24). No PPV added (1906.68 vs invoice 1828.08). Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -927,7 +927,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58383 (prototype vendor Marmon-Keystone; only historical receipt already invoiced). Did not invent lines. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58383 (prototype vendor Marmon-Keystone; only historical receipt already invoiced). Did not invent lines. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -985,7 +985,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: slip 331201 two A-02393-000 qty 42+42 plus A-09128-000* lid qty 30. Skipped 8/4 and negative qty. Amount 13404.84 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: slip 331201 two A-02393-000 qty 42+42 plus A-09128-000* lid qty 30. Skipped 8/4 and negative qty. Amount 13404.84 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58799 PL-0.25 X 60 X 120-A572 qty 5 slip 84615375. No $0 freight charge. Amount 2278.11 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: PO58799 PL-0.25 X 60 X 120-A572 qty 5 slip 84615375. No $0 freight charge. Amount 2278.11 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: only 8/3 slip 84623830 TP-0.125 x 60 x 120-A36 qty 20. Did not select 8/5 PL-0.375. Amount 5580.96 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: only 8/3 slip 84623830 TP-0.125 x 60 x 120-A36 qty 20. Did not select 8/5 PL-0.375. Amount 5580.96 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 15 PO58749 receipts. Posted F-Fees &amp; Surcharges 124.83 Shipping &amp; Handling (not PPV). Amount 2620.08 matches. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: all 15 PO58749 receipts. Posted F-Fees &amp; Surcharges 124.83 Shipping &amp; Handling (not PPV). Amount 2620.08 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 3 PO58764 receipts slips TXFT499769. Posted F-Fees &amp; Surcharges 122.69 Shipping &amp; Handling (not PPV). Amount 424.89 vs verification 424.88. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: all 3 PO58764 receipts slips TXFT499769. Posted F-Fees &amp; Surcharges 122.69 Shipping &amp; Handling (not PPV). Amount 424.89 vs verification 424.88. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58821. Did not invent freight 700. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58821. Did not invent freight 700. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58717. Did not invent freight 500. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58717. Did not invent freight 500. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58742. Did not invent freight 200. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>HOLD-no-receipts. Select Receipts empty for PO 58742. Did not invent freight 200. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both PO58814 receipts slip G62282. Posted F-Fees &amp; Surcharges 60.00 SHIPPING &amp; HANDLING SURCHARGE (not PPV). Amount 1681.19 vs verification 1681.31. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: both PO58814 receipts slip G62282. Posted F-Fees &amp; Surcharges 60.00 SHIPPING &amp; HANDLING SURCHARGE (not PPV). Amount 1681.19 vs verification 1681.31. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both PO58810 RB-4.00-6061 receipts 13+35 slip S812773. Amount 393.60 vs verification 393.62. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: both PO58810 RB-4.00-6061 receipts 13+35 slip S812773. Amount 393.60 vs verification 393.62. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58723-02 qty 1 and PO58723-03 qty 2. Did not Add Item for unreceived line 01. Posted F-Fees &amp; Surcharges 12.40 Packaging/Shop Supplies Recovery (NOT PPV). Amount 670.36 vs verification 1252.18. Attach=login-blocked: OUTLOOK_AP_PASSWORD present but Microsoft rejected it for accountspayable@kannonmfg.com (incorrect account or password). OUTLOOK_AP_USERNAME is present but is not that mailbox so it was not used. MICROSOFT_GRAPH_* absent. No other mailbox opened. No PDF downloaded.</t>
+          <t>Select Receipts: PO58723-02 qty 1 and PO58723-03 qty 2. Did not Add Item for unreceived line 01. Posted F-Fees &amp; Surcharges 12.40 Packaging/Shop Supplies Recovery (NOT PPV). Amount 670.36 vs verification 1252.18. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>login-blocked</t>
+          <t>attached</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record no-PO batch 671 headers 9500-9507 and Graph attaches
Eight Miscellaneous AP headers created with Purchase Order blank.
PDFs pulled from accountspayable@kannonmfg.com and attached via
the prototype paperclip. ENGIE and Waste Connections stay HOLD
(no existing vendor/remit/terms). CHECK STOP stays HOLD. GRM
00012913 already exists as id 3854. 9481-9499 untouched.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -54,6 +54,11 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -67,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -79,6 +84,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1654,7 +1662,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no-PO. No-PO invoices do not get a header.</t>
+          <t>HOLD: vendor/remit/terms not found on prototype for ENGIE Resources LLC. No existing ENGIE AP invoice to copy from; will not invent vendor/remit/terms.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -1675,7 +1683,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-header</t>
         </is>
       </c>
     </row>
@@ -1699,17 +1707,19 @@
       <c r="E22" s="2" t="n">
         <v>2391.09</v>
       </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no-PO. No-PO invoices do not get a header.</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>9500</v>
+      </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
           <t>API Agent - 8/27/26 (671)</t>
@@ -1727,7 +1737,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1751,17 +1761,19 @@
       <c r="E23" s="2" t="n">
         <v>744.5</v>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no-PO. No-PO invoices do not get a header.</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>9501</v>
+      </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
           <t>API Agent - 8/27/26 (671)</t>
@@ -1779,7 +1791,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1803,17 +1815,19 @@
       <c r="E24" s="2" t="n">
         <v>814.73</v>
       </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no-PO. No-PO invoices do not get a header.</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>9502</v>
+      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>API Agent - 8/27/26 (671)</t>
@@ -1831,7 +1845,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1855,17 +1869,19 @@
       <c r="E25" s="2" t="n">
         <v>997.34</v>
       </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no-PO. No-PO invoices do not get a header.</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Energy surcharge + garment protection fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>9503</v>
+      </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
           <t>API Agent - 8/27/26 (671)</t>
@@ -1883,7 +1899,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -1907,17 +1923,19 @@
       <c r="E26" s="2" t="n">
         <v>189.78</v>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no-PO. No-PO invoices do not get a header.</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr"/>
+          <t>Fail/already exists (id 3854 is Precision Fabrication, not GRM). Did not recreate per invoice-number rule.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>3854</v>
+      </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
           <t>API Agent - 8/27/26 (671)</t>
@@ -1935,7 +1953,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>not-attempted</t>
         </is>
       </c>
     </row>
@@ -1959,17 +1977,19 @@
       <c r="E27" s="2" t="n">
         <v>1694.48</v>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no-PO. No-PO invoices do not get a header.</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>9504</v>
+      </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
           <t>API Agent - 8/27/26 (671)</t>
@@ -1987,7 +2007,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2038,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no-PO. No-PO invoices do not get a header.</t>
+          <t>HOLD: vendor/remit/terms not found on prototype for Waste Connections Lone Star, Inc. No existing Waste Connections AP invoice to copy from; will not invent vendor/remit/terms. PDF is in AP mailbox.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -2039,7 +2059,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-header</t>
         </is>
       </c>
     </row>
@@ -2063,17 +2083,19 @@
       <c r="E29" s="2" t="n">
         <v>840</v>
       </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no-PO. No-PO invoices do not get a header.</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>9506</v>
+      </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
           <t>API Agent - 8/27/26 (671)</t>
@@ -2091,7 +2113,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -2115,17 +2137,19 @@
       <c r="E30" s="2" t="n">
         <v>485.7</v>
       </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no-PO. No-PO invoices do not get a header.</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Freight Charge 485.70 goes to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>9507</v>
+      </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
           <t>API Agent - 8/27/26 (671)</t>
@@ -2143,7 +2167,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2219,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>no-header</t>
         </is>
       </c>
     </row>
@@ -2219,17 +2243,19 @@
       <c r="E32" s="2" t="n">
         <v>1463.98</v>
       </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>HOLD: no-PO. No-PO invoices do not get a header.</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
+          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Rental + fuel surcharge go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>9505</v>
+      </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>API Agent - 8/27/26 (671)</t>
@@ -2247,7 +2273,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>attached</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record first live AP run: batch 688, headers 9663-9677, Excel report.
20 mailbox invoices attempted on live.kimcoerp.com. 15 Success, 5 Fail, 0 HOLD. Outlook was not flagged. Attach notify was 405. Report is runs/AP-run-2026-08-27.xlsx.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -10,7 +10,7 @@
     <sheet name="AP run" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$L$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$M$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,11 +47,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -72,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -84,9 +79,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -454,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -469,6 +461,7 @@
     <col width="40" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -532,30 +525,35 @@
           <t>Attach status</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Flag in Outlook</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Telecom Products Inc.</t>
+          <t>TELECOM PRODUCTS INC.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>16960</t>
+          <t>17601</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>58351</t>
+          <t>58514</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>10431.36</v>
+        <v>1738.56</v>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
@@ -564,15 +562,15 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: slip 106081 qty 38+58=96 of A-04421-000 @ 108.66. Invoice amount 10431.36 matches. No fees. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>9481</v>
+        <v>9663</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -587,33 +585,34 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>McMaster-Carr Supply Company</t>
+          <t>RMP Industrial Supply Inc</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>69233267</t>
+          <t>1472035</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>58808</t>
-        </is>
-      </c>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="n">
-        <v>489.14</v>
+        <v>59.39</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
@@ -622,20 +621,20 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: 5913K74 qty 10 and 91263A232 qty 5. Did not Add Item for unreceived 8701K65. Posted F-Fees &amp; Surcharges 42.17 Shipping (not PPV). Amount 205.52 vs verification 489.14 because line 01 has no receipt. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>9482</v>
+        <v>9664</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Shipping 42.17</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -645,33 +644,34 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>McMaster-Carr Supply Company</t>
+          <t>Tejas Transportation</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>69313216</t>
+          <t>523856</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>58826</t>
-        </is>
-      </c>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="n">
-        <v>467.22</v>
+        <v>400</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
@@ -680,20 +680,20 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 8 PO58826 receipts slip 3262728-02. Posted F-Fees &amp; Surcharges 38.83 Shipping (not PPV). Amount 467.22 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>9483</v>
+        <v>9665</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Shipping 38.83</t>
+          <t>1. Transport freight to KT Galvanizing- Venus, TX 1 $250.00 250.00; 2. Return freight to Kannon 1 $150.00 150.00</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -703,33 +703,34 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Purvis Industries Ft Worth</t>
+          <t>Air Products and Chemicals, Inc</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>32605959</t>
+          <t>436251638</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>58556</t>
-        </is>
-      </c>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="n">
-        <v>480.05</v>
+        <v>2017.2</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
@@ -738,20 +739,20 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58556-01 qty 10 slip 23016800. Posted F-Fees &amp; Surcharges 27.12 Total Freight In (not PPV). Amount 480.05 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>9484</v>
+        <v>9666</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Total Freight In 27.12</t>
+          <t>Product Surcharge 6.67; The total amount due from the customer may include various itemized charges, inc; hazardous materials; charges for handling, delivery, and shipping; and/or charge</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -761,55 +762,60 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Capital Machine Technologies, Inc</t>
+          <t>Earle M. Jorgensen Co</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>26167</t>
+          <t>S814379432</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>58634</t>
+          <t>58984</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>403</v>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>752.1</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Did not invent lines or freight. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>9485</v>
+        <v>9667</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Freight (UPS) 34.00</t>
+          <t>SHIPPING DATE 26-AUG-2026; FREIGHT PAYMENT PREPAID</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -819,55 +825,60 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Capital Machine Technologies, Inc</t>
+          <t>O'Neal Steel - Dallas (GP)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>26258</t>
+          <t>15452509</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>58634</t>
+          <t>59028</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>940</v>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>670.7</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58634. Shop supplies 25.00 would be F-Fees &amp; Surcharges never PPV, but no receipts so no invented lines/charges. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>9486</v>
+        <v>9668</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>SUPPLY FEE / Shop supplies 25.00</t>
+          <t>Total Freight: .00; Shipped Via Freight Handling Code</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -877,33 +888,34 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Willbanks Metals Inc</t>
+          <t>Gas and Supply North Texas, LLC</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>209661</t>
+          <t>0040386181</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>58504</t>
-        </is>
-      </c>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="n">
-        <v>1828.08</v>
+        <v>144</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
@@ -912,15 +924,15 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both 7/30 slip 186040-3 (S0264-1 qty 12, S0264-4 qty 24). No PPV added (1906.68 vs invoice 1828.08). Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>9487</v>
+        <v>9669</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -935,55 +947,60 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Willbanks Metals Inc</t>
+          <t>McMaster-Carr Supply Company</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>209664</t>
+          <t>70846521</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>58383</t>
+          <t>59045</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3347.97</v>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>1247.28</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58383 (prototype vendor Marmon-Keystone; only historical receipt already invoiced). Did not invent lines. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>9488</v>
+        <v>9670</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Shipping 68.93</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -993,33 +1010,34 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Morgan Steel LLC</t>
+          <t>Luxor Staffing, Inc.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>128269</t>
+          <t>364459</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>58718</t>
-        </is>
-      </c>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="n">
-        <v>13404.84</v>
+        <v>3139.5</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
@@ -1028,15 +1046,15 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: slip 331201 two A-02393-000 qty 42+42 plus A-09128-000* lid qty 30. Skipped 8/4 and negative qty. Amount 13404.84 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>9489</v>
+        <v>9671</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1051,55 +1069,58 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>O'Neal Steel - Dallas (GP)</t>
+          <t>National Specialty Alloys, Inc</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>15423965</t>
+          <t>453743</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>58799</t>
+          <t>58978</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2278.11</v>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+        <v>118</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58799 PL-0.25 X 60 X 120-A572 qty 5 slip 84615375. No $0 freight charge. Amount 2278.11 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>9490</v>
-      </c>
+          <t>Fail: vendor missing on live for National Specialty Alloys, Inc (PO 58978 exists as PO58978-National Specialty Alloys). Will not invent a vendor/remit-to ID.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Freight 0.00</t>
+          <t>Please note that there will be a 2.6% surcharge applied to all credit card trans</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1109,33 +1130,38 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>no-pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>O'Neal Steel - Dallas (GP)</t>
+          <t>Modern Heat Treat Inc</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>15427085</t>
+          <t>220804</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>58831</t>
+          <t>58934</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>5580.96</v>
+        <v>201.25</v>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
@@ -1144,20 +1170,20 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: only 8/3 slip 84623830 TP-0.125 x 60 x 120-A36 qty 20. Did not select 8/5 PL-0.375. Amount 5580.96 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>9491</v>
+        <v>9672</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Freight 0.00</t>
+          <t>$26.25Surcharge 26.25</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1167,33 +1193,38 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Fastenal Company</t>
+          <t>TELECOM PRODUCTS INC.</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>TXFT499739</t>
+          <t>17602</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>58749</t>
+          <t>58736</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>2620.08</v>
+        <v>6954.24</v>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
@@ -1202,20 +1233,20 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 15 PO58749 receipts. Posted F-Fees &amp; Surcharges 124.83 Shipping &amp; Handling (not PPV). Amount 2620.08 matches. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>9492</v>
+        <v>9673</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Shipping &amp; Handling 124.83</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1225,7 +1256,12 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1237,43 +1273,43 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>TXFT499769</t>
+          <t>TXFT496725</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>58764</t>
+          <t>56787</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>424.88</v>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+        <v>357.35</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: all 3 PO58764 receipts slips TXFT499769. Posted F-Fees &amp; Surcharges 122.69 Shipping &amp; Handling (not PPV). Amount 424.89 vs verification 424.88. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Fail/already exists (id 6488)</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>9493</v>
+        <v>6488</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Shipping &amp; Handling 122.69</t>
+          <t>1 1 0 FREIGHT CHARGE FHTX18656 90000001 17,500.0000 175.00 N2 175.00; Shipping &amp; Handling</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1283,55 +1319,60 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>no-pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Legacy Wire Products</t>
+          <t>Fastenal Company</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>PS-INV103935</t>
+          <t>TXFT499726</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>58821</t>
+          <t>58732</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>2545</v>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>296.59</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58821. Did not invent freight 700. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>9494</v>
+        <v>9674</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Freight Charge 700.00</t>
+          <t>Shipping &amp; Handling</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1341,55 +1382,60 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Legacy Wire Products</t>
+          <t>Fastenal Company</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>PS-INV103936</t>
+          <t>TXFT499646</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>58717</t>
+          <t>58707</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>2140</v>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>78.19</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58717. Did not invent freight 500. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>9495</v>
+        <v>9675</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Freight Charge 500.00</t>
+          <t>Shipping &amp; Handling</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1399,55 +1445,60 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Legacy Wire Products</t>
+          <t>Fastenal Company</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>PS-INV103937</t>
+          <t>TXFT499639</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>58742</t>
+          <t>58692</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>856</v>
+        <v>92.17</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>HOLD-no-receipts. Select Receipts empty for PO 58742. Did not invent freight 200. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Fail/already exists (id 9642)</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>9496</v>
+        <v>9642</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Freight Charge 200.00</t>
+          <t>Shipping &amp; Handling</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1457,33 +1508,38 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>no-pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Eastern Metal Supply of Texas, LLC</t>
+          <t>Fastenal Company</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>816292</t>
+          <t>TXFT499357</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>58814</t>
+          <t>58462</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>1681.31</v>
+        <v>134.86</v>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
@@ -1492,20 +1548,20 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both PO58814 receipts slip G62282. Posted F-Fees &amp; Surcharges 60.00 SHIPPING &amp; HANDLING SURCHARGE (not PPV). Amount 1681.19 vs verification 1681.31. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>9497</v>
+        <v>9676</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>SHIPPING &amp; HANDLING SURCHARGE 60.00</t>
+          <t>Shipping &amp; Handling</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1515,33 +1571,38 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Earle M. Jorgensen Co</t>
+          <t>Fastenal Company</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>S812773432</t>
+          <t>TXFT499356</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>58810</t>
+          <t>58015</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>393.62</v>
+        <v>19.8</v>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
@@ -1550,20 +1611,20 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: both PO58810 RB-4.00-6061 receipts 13+35 slip S812773. Amount 393.60 vs verification 393.62. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>9498</v>
+        <v>9677</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Shipping &amp; Handling</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1573,55 +1634,60 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>blocked-405</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Crosslink Powder Coating of TX, LLC</t>
+          <t>Fastenal Company</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>27756</t>
+          <t>TXFT499528</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>58723</t>
+          <t>58603</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1252.18</v>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
+        <v>1798.53</v>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts: PO58723-02 qty 1 and PO58723-03 qty 2. Did not Add Item for unreceived line 01. Posted F-Fees &amp; Surcharges 12.40 Packaging/Shop Supplies Recovery (NOT PPV). Amount 670.36 vs verification 1252.18. Attach=attached: PDF pulled via Microsoft Graph from accountspayable@kannonmfg.com only (client-credentials; no other mailbox queried) and uploaded on the invoice HEADER (paperclip tab → Upload → Save). Bills were not voided/deleted/recreated.</t>
+          <t>Fail/already exists (id 9444)</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>9499</v>
+        <v>9444</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Packaging/Shop Supplies Recovery 12.40</t>
+          <t>Shipping &amp; Handling</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1631,49 +1697,58 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>attached</t>
+          <t>no-pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ENGIE Resources LLC</t>
+          <t>Coherent Corp.</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>11367279</t>
+          <t>120953</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>58886</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="n">
-        <v>416.1</v>
+        <v>790.65</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>HOLD: vendor/remit/terms not found on prototype for ENGIE Resources LLC. No existing ENGIE AP invoice to copy from; will not invent vendor/remit/terms.</t>
+          <t>Fail: vendor missing on live for Coherent Corp. (PO 58886 exists as PO58886-Coherent Corp.). Will not invent a vendor/remit-to ID.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 8/27/26 (671)</t>
+          <t>API Agent - 8/27/26 (688)</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Incremental System Admin Fee 0.20; Market Securitization 1.44; Settlement 1.64; Taxes/Fees 8.79</t>
+          <t>SHIPPING REFERENCE; 2 9308027 INTERNATIONAL TRADE SURCHARGE - IR SAX, PO_LINE_NUMBER: 1 1 37.65 37.65; SUBTOTAL SHIPPING/HANDLING TAX TOTAL</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1683,602 +1758,17 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>no-header</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Hudson Energy Services, LLC</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>2608001907</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="n">
-        <v>2391.09</v>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>9500</v>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>API Agent - 8/27/26 (671)</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>ERCOT/market/TDSP pass-throughs</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>attached</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>UniFirst First Aid &amp; Safety</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>42203000308</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="n">
-        <v>744.5</v>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>9501</v>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>API Agent - 8/27/26 (671)</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>attached</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Shoppa's Material Handling, Ltd</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>PSI-001216291</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="n">
-        <v>814.73</v>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>9502</v>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>API Agent - 8/27/26 (671)</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>attached</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>UniFirst Corporation</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>2810786878</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="2" t="n">
-        <v>997.34</v>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Energy surcharge + garment protection fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>9503</v>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>API Agent - 8/27/26 (671)</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>Energy Surcharge 3.00; garment protection fees</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>attached</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>GRM Information Management Services of Dallas, LLC</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>00012913</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="n">
-        <v>189.78</v>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>Fail/already exists (id 3854 is Precision Fabrication, not GRM). Did not recreate per invoice-number rule.</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>3854</v>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>API Agent - 8/27/26 (671)</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>Account Maintenance 22.68; Check Processing 25.00</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>not-attempted</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>NTEX Electric Inc.</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>17-2557</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="2" t="n">
-        <v>1694.48</v>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>9504</v>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>API Agent - 8/27/26 (671)</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>attached</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Waste Connections Lone Star, Inc</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>3485086V190</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="n">
-        <v>357.8</v>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>HOLD: vendor/remit/terms not found on prototype for Waste Connections Lone Star, Inc. No existing Waste Connections AP invoice to copy from; will not invent vendor/remit/terms. PDF is in AP mailbox.</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>API Agent - 8/27/26 (671)</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>no-header</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Luxor Staffing, Inc.</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>361804</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="2" t="n">
-        <v>840</v>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Fees go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="n">
-        <v>9506</v>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>API Agent - 8/27/26 (671)</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>attached</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Priority1</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>17840758</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="n">
-        <v>485.7</v>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Freight Charge 485.70 goes to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="n">
-        <v>9507</v>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>API Agent - 8/27/26 (671)</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>Freight Charge 485.70</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>attached</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Gas and Supply North Texas, LLC</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>0040325801</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="2" t="n">
-        <v>418.93</v>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>HOLD: CHECK STOP. Do not create a header.</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>API Agent - 8/27/26 (671)</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>FUEL SURCHARGE 17.50</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>no-header</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Gas and Supply North Texas, LLC</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>0040333419</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="n">
-        <v>1463.98</v>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>Header created (Invoice_Type 4 Miscellaneous). Purchase Order left blank. Do not Select Receipts or invent PO lines. Rental + fuel surcharge go to F-Fees &amp; Surcharges (not PPV). Graph+GUI paperclip attached.</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="n">
-        <v>9505</v>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>API Agent - 8/27/26 (671)</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>rental + fuel surcharge</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>attached</t>
+          <t>no-pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L32"/>
+  <autoFilter ref="A1:M21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record live Select Receipts and PDF attaches on 9663-9677.
GUI work on the existing batch 688 Success headers only. 9/10 PO bills had receipts selected; Fastenal TXFT499356 is HOLD-no-receipts. All 15 vendor PDFs attached. Fees posted as F-Fees & Surcharges; PPV only on TXFT499646. Outlook not flagged. Fail rows unchanged.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>Select Receipts done: slip 106620 qty 16 (did not take 8/5 qty 84). Lines 1738.56 match verification. No fee. No PPV. PDF attached. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -575,17 +575,17 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
+          <t>none posted</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
           <t>none</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only. No Add Item. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -634,17 +634,17 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
+          <t>none posted</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
           <t>none</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only. Freight stays on the vendor bill; no typed lines. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -693,7 +693,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>1. Transport freight to KT Galvanizing- Venus, TX 1 $250.00 250.00; 2. Return freight to Kannon 1 $150.00 150.00</t>
+          <t>none posted (no-PO attach-only)</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only. Delivery/hazmat/surcharge left on the bill; no Add Item. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -752,7 +752,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Product Surcharge 6.67; The total amount due from the customer may include various itemized charges, inc; hazardous materials; charges for handling, delivery, and shipping; and/or charge</t>
+          <t>none posted (no-PO attach-only)</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>Select Receipts done: matching slip S814379 part RB-1.25-1018. Line extended 770.16 vs invoice 752.10 (receipt qty 1147.1 vs billed 752.10; UOM/weight, not a unit-price gap). No PPV posted. Freight prepaid. PDF attached. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -815,17 +815,17 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>SHIPPING DATE 26-AUG-2026; FREIGHT PAYMENT PREPAID</t>
+          <t>none posted (freight prepaid)</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>none (qty/UOM gap, not unit price)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>Select Receipts done: slip 84687574 qty 2400. Line 670.80 vs invoice 670.70 ($0.10 rounding). No fee. No PPV. PDF attached. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -878,17 +878,17 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Total Freight: .00; Shipped Via Freight Handling Code</t>
+          <t>none posted (freight .00)</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>none ($0.10 rounding)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only (invoice 0040386181 in vendor file). No Add Item. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -937,17 +937,17 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
+          <t>none posted</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
           <t>none</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>Select Receipts done: all 5 receipts slip 4652696-01. Additional Charge F-Fees &amp; Surcharges 68.93 Shipping posted (not PPV). Lines 1178.35 + fee 68.93 = 1247.28. PDF attached. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Shipping 68.93</t>
+          <t>F-Fees &amp; Surcharges 68.93 Shipping (posted)</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 4). Purchase Order left blank (no-PO or multi-PO or PO not on target). Do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>No-PO Type 4. Select Receipts not applicable. PDF attached: KANNON 364459 only (timesheet 8.23 not attached). No Add Item. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -1059,17 +1059,17 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
+          <t>none posted</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
           <t>none</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>Select Receipts done: slip 220654 qty 2+4+2 only (did not take slip 220655). Additional Charge F-Fees &amp; Surcharges 26.25 Surcharge posted (not PPV). Lines 174.96 + 26.25 = 201.21 vs verification 201.25. PDF attached. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>$26.25Surcharge 26.25</t>
+          <t>F-Fees &amp; Surcharges 26.25 Surcharge (posted)</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>Select Receipts done: slip 106621 qty 64 (did not take 8/26 qty 36). Lines 6954.24 match verification. No fee. PDF attached. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
+          <t>none posted</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
           <t>none</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>Select Receipts done: slip txft499726 qty 300. Additional Charge F-Fees &amp; Surcharges 92.05 Shipping &amp; Handling posted (not PPV). Lines 204.54 + 92.05 = 296.59. PDF attached. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Shipping &amp; Handling</t>
+          <t>F-Fees &amp; Surcharges 92.05 Shipping &amp; Handling (posted)</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>Select Receipts done: slip TXFT499646 qty 120. Posted F-Fees &amp; Surcharges 21.79 Shipping &amp; Handling and Purchase Price Variance 4.80 (invoice merch 56.40 vs PO 51.60 = 6.1% of invoice total, under 10%). Lines 51.60 + 26.59 = 78.19. PDF attached. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1435,17 +1435,17 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Shipping &amp; Handling</t>
+          <t>F-Fees &amp; Surcharges 21.79 Shipping &amp; Handling (posted)</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>PPV 4.80 posted (unit price 0.47 vs PO 0.43)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>Select Receipts done: five slip TXFT499357 rows qty 10+20+4+4+8=46 (did not take TXFT499392). Additional Charge F-Fees &amp; Surcharges 21.70 Shipping &amp; Handling posted (not PPV). Lines 113.16 + 21.70 = 134.86. PDF attached. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Shipping &amp; Handling</t>
+          <t>F-Fees &amp; Surcharges 21.70 Shipping &amp; Handling (posted)</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Header created (Invoice_Type 3). Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Fees go to Additional Charge Fees and surcharges / F-Fees &amp; Surcharges (not PPV). Attach status=blocked-405.</t>
+          <t>HOLD-no-receipts: invoice qty 6 of 50006-5 / 99472056; no live receipt has slip TXFT499356 or qty 6. Did not guess other slips. Shipping 5.04 not posted. PDF attached. Outlook not flagged.</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Shipping &amp; Handling</t>
+          <t>none posted (HOLD-no-receipts)</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>blocked-405</t>
+          <t>attached</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Use preexisting Entered in AI category as the Outlook process marker.
Apply Entered in AI to 14 already-Success 8/27 AP messages. Remove AP Matched and clear the follow-up flag on Telecom 17601. Skip HOLD/Fail. CLI no longer PATCHes flag.flagStatus.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-08-27.xlsx
+++ b/runs/AP-run-2026-08-27.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -462,6 +462,7 @@
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -530,6 +531,11 @@
           <t>Flag in Outlook</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Flag status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -562,7 +568,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts done: slip 106620 qty 16 (did not take 8/5 qty 84). Lines 1738.56 match verification. No fee. No PPV. PDF attached. Outlook not flagged.</t>
+          <t>Select Receipts done: slip 106620 qty 16 (did not take 8/5 qty 84). Lines 1738.56 match verification. No fee. No PPV. PDF attached. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -591,6 +597,11 @@
       <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -621,7 +632,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only. No Add Item. Outlook not flagged.</t>
+          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only. No Add Item. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -650,6 +661,11 @@
       <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -680,7 +696,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only. Freight stays on the vendor bill; no typed lines. Outlook not flagged.</t>
+          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only. Freight stays on the vendor bill; no typed lines. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -709,6 +725,11 @@
       <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -739,7 +760,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only. Delivery/hazmat/surcharge left on the bill; no Add Item. Outlook not flagged.</t>
+          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only. Delivery/hazmat/surcharge left on the bill; no Add Item. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -770,6 +791,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -802,7 +828,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts done: matching slip S814379 part RB-1.25-1018. Line extended 770.16 vs invoice 752.10 (receipt qty 1147.1 vs billed 752.10; UOM/weight, not a unit-price gap). No PPV posted. Freight prepaid. PDF attached. Outlook not flagged.</t>
+          <t>Select Receipts done: matching slip S814379 part RB-1.25-1018. Line extended 770.16 vs invoice 752.10 (receipt qty 1147.1 vs billed 752.10; UOM/weight, not a unit-price gap). No PPV posted. Freight prepaid. PDF attached. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -833,6 +859,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -865,7 +896,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts done: slip 84687574 qty 2400. Line 670.80 vs invoice 670.70 ($0.10 rounding). No fee. No PPV. PDF attached. Outlook not flagged.</t>
+          <t>Select Receipts done: slip 84687574 qty 2400. Line 670.80 vs invoice 670.70 ($0.10 rounding). No fee. No PPV. PDF attached. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -894,6 +925,11 @@
       <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -924,7 +960,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only (invoice 0040386181 in vendor file). No Add Item. Outlook not flagged.</t>
+          <t>No-PO Type 4. Select Receipts not applicable. PDF attached only (invoice 0040386181 in vendor file). No Add Item. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -955,6 +991,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -987,7 +1028,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts done: all 5 receipts slip 4652696-01. Additional Charge F-Fees &amp; Surcharges 68.93 Shipping posted (not PPV). Lines 1178.35 + fee 68.93 = 1247.28. PDF attached. Outlook not flagged.</t>
+          <t>Select Receipts done: all 5 receipts slip 4652696-01. Additional Charge F-Fees &amp; Surcharges 68.93 Shipping posted (not PPV). Lines 1178.35 + fee 68.93 = 1247.28. PDF attached. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -1016,6 +1057,11 @@
       <c r="M9" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1092,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>No-PO Type 4. Select Receipts not applicable. PDF attached: KANNON 364459 only (timesheet 8.23 not attached). No Add Item. Outlook not flagged.</t>
+          <t>No-PO Type 4. Select Receipts not applicable. PDF attached: KANNON 364459 only (timesheet 8.23 not attached). No Add Item. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -1077,6 +1123,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1138,6 +1189,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>skipped-not-success</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1170,7 +1226,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts done: slip 220654 qty 2+4+2 only (did not take slip 220655). Additional Charge F-Fees &amp; Surcharges 26.25 Surcharge posted (not PPV). Lines 174.96 + 26.25 = 201.21 vs verification 201.25. PDF attached. Outlook not flagged.</t>
+          <t>Select Receipts done: slip 220654 qty 2+4+2 only (did not take slip 220655). Additional Charge F-Fees &amp; Surcharges 26.25 Surcharge posted (not PPV). Lines 174.96 + 26.25 = 201.21 vs verification 201.25. PDF attached. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -1201,6 +1257,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1233,7 +1294,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts done: slip 106621 qty 64 (did not take 8/26 qty 36). Lines 6954.24 match verification. No fee. PDF attached. Outlook not flagged.</t>
+          <t>Select Receipts done: slip 106621 qty 64 (did not take 8/26 qty 36). Lines 6954.24 match verification. No fee. PDF attached. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -1264,6 +1325,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1327,6 +1393,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>skipped-not-success</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1359,7 +1430,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts done: slip txft499726 qty 300. Additional Charge F-Fees &amp; Surcharges 92.05 Shipping &amp; Handling posted (not PPV). Lines 204.54 + 92.05 = 296.59. PDF attached. Outlook not flagged.</t>
+          <t>Select Receipts done: slip txft499726 qty 300. Additional Charge F-Fees &amp; Surcharges 92.05 Shipping &amp; Handling posted (not PPV). Lines 204.54 + 92.05 = 296.59. PDF attached. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -1390,6 +1461,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1422,7 +1498,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts done: slip TXFT499646 qty 120. Posted F-Fees &amp; Surcharges 21.79 Shipping &amp; Handling and Purchase Price Variance 4.80 (invoice merch 56.40 vs PO 51.60 = 6.1% of invoice total, under 10%). Lines 51.60 + 26.59 = 78.19. PDF attached. Outlook not flagged.</t>
+          <t>Select Receipts done: slip TXFT499646 qty 120. Posted F-Fees &amp; Surcharges 21.79 Shipping &amp; Handling and Purchase Price Variance 4.80 (invoice merch 56.40 vs PO 51.60 = 6.1% of invoice total, under 10%). Lines 51.60 + 26.59 = 78.19. PDF attached. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1453,6 +1529,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1516,6 +1597,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>skipped-not-success</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1548,7 +1634,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Select Receipts done: five slip TXFT499357 rows qty 10+20+4+4+8=46 (did not take TXFT499392). Additional Charge F-Fees &amp; Surcharges 21.70 Shipping &amp; Handling posted (not PPV). Lines 113.16 + 21.70 = 134.86. PDF attached. Outlook not flagged.</t>
+          <t>Select Receipts done: five slip TXFT499357 rows qty 10+20+4+4+8=46 (did not take TXFT499392). Additional Charge F-Fees &amp; Surcharges 21.70 Shipping &amp; Handling posted (not PPV). Lines 113.16 + 21.70 = 134.86. PDF attached. Outlook not flagged. Outlook category Entered in AI applied; follow-up flag not used.</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1579,6 +1665,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1639,7 +1730,12 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>skipped-hold-no-receipts</t>
         </is>
       </c>
     </row>
@@ -1705,6 +1801,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>skipped-not-success</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1764,6 +1865,11 @@
       <c r="M21" s="2" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>skipped-not-success</t>
         </is>
       </c>
     </row>

</xml_diff>